<commit_message>
Update Increase By Realitive Increase (n=previous n + n-1).xlsx
</commit_message>
<xml_diff>
--- a/Increase By Realitive Increase (n=previous n + n-1).xlsx
+++ b/Increase By Realitive Increase (n=previous n + n-1).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30126"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0ECAD8CF-EA2D-4EF1-AD3C-EFB90A6214E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F980FECF-1044-47EF-8D26-922B5452EAD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Iteration</t>
   </si>
@@ -49,6 +49,9 @@
   </si>
   <si>
     <t>Z (Previous Z + Y)</t>
+  </si>
+  <si>
+    <t>Base Value</t>
   </si>
 </sst>
 </file>
@@ -90,7 +93,11 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -108,8 +115,8 @@
   <autoFilter ref="A1:E11" xr:uid="{C0C2D9BF-77A2-4416-A812-86AF040207A5}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{B1013B72-9008-4CDB-803D-7509B6F3B922}" name="Iteration"/>
-    <tableColumn id="2" xr3:uid="{02179467-1A22-4FBD-B0E6-4A7F8563D6B2}" name="I (initial value)">
-      <calculatedColumnFormula>1</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{02179467-1A22-4FBD-B0E6-4A7F8563D6B2}" name="I (initial value)" dataDxfId="0">
+      <calculatedColumnFormula>$H$2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{1292F0F5-19F3-4372-9149-F457D83BA48B}" name="X (previous X + I)">
       <calculatedColumnFormula>IF(ISNUMBER(C1),C1,0)+B2</calculatedColumnFormula>
@@ -422,13 +429,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -444,215 +451,221 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
-        <f>1</f>
-        <v>1</v>
+        <f t="shared" ref="B2:B11" si="0">$H$2</f>
+        <v>5</v>
       </c>
       <c r="C2">
         <f>IF(ISNUMBER(C1),C1,0)+B2</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <f>IF(ISNUMBER(D1),D1,0)+C2</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <f>IF(ISNUMBER(E1),E1,0)+D2</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>5</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <f>1</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="C3">
         <f>IF(ISNUMBER(C2),C2,0)+B3</f>
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D3">
         <f>IF(ISNUMBER(D2),D2,0)+C3</f>
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E3">
         <f>IF(ISNUMBER(E2),E2,0)+D3</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <f>1</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="C4">
         <f>IF(ISNUMBER(C3),C3,0)+B4</f>
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="D4">
         <f>IF(ISNUMBER(D3),D3,0)+C4</f>
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="E4">
         <f>IF(ISNUMBER(E3),E3,0)+D4</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
-        <f>1</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="C5">
         <f>IF(ISNUMBER(C4),C4,0)+B5</f>
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D5">
         <f>IF(ISNUMBER(D4),D4,0)+C5</f>
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E5">
         <f>IF(ISNUMBER(E4),E4,0)+D5</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
-        <f>1</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="C6">
         <f>IF(ISNUMBER(C5),C5,0)+B6</f>
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="D6">
         <f>IF(ISNUMBER(D5),D5,0)+C6</f>
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="E6">
         <f>IF(ISNUMBER(E5),E5,0)+D6</f>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
-        <f>1</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="C7">
         <f>IF(ISNUMBER(C6),C6,0)+B7</f>
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="D7">
         <f>IF(ISNUMBER(D6),D6,0)+C7</f>
-        <v>21</v>
+        <v>105</v>
       </c>
       <c r="E7">
         <f>IF(ISNUMBER(E6),E6,0)+D7</f>
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
-        <f>1</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="C8">
         <f>IF(ISNUMBER(C7),C7,0)+B8</f>
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="D8">
         <f>IF(ISNUMBER(D7),D7,0)+C8</f>
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="E8">
         <f>IF(ISNUMBER(E7),E7,0)+D8</f>
-        <v>84</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
-        <f>1</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="C9">
         <f>IF(ISNUMBER(C8),C8,0)+B9</f>
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="D9">
         <f>IF(ISNUMBER(D8),D8,0)+C9</f>
-        <v>36</v>
+        <v>180</v>
       </c>
       <c r="E9">
         <f>IF(ISNUMBER(E8),E8,0)+D9</f>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
-        <f>1</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="C10">
         <f>IF(ISNUMBER(C9),C9,0)+B10</f>
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="D10">
         <f>IF(ISNUMBER(D9),D9,0)+C10</f>
-        <v>45</v>
+        <v>225</v>
       </c>
       <c r="E10">
         <f>IF(ISNUMBER(E9),E9,0)+D10</f>
-        <v>165</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
-        <f>1</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="C11">
         <f>IF(ISNUMBER(C10),C10,0)+B11</f>
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="D11">
         <f>IF(ISNUMBER(D10),D10,0)+C11</f>
-        <v>55</v>
+        <v>275</v>
       </c>
       <c r="E11">
         <f>IF(ISNUMBER(E10),E10,0)+D11</f>
-        <v>220</v>
+        <v>1100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>